<commit_message>
fix: synthetic datasets generator fix
</commit_message>
<xml_diff>
--- a/data/planning/duplicate_coordinates.xlsx
+++ b/data/planning/duplicate_coordinates.xlsx
@@ -3243,50 +3243,85 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>work_type_id</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>received_at</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>sla_deadline_at</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>required_transport_type</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>service_duration_source</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>status</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>visit_window_start</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>visit_window_end</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>planned_start_at</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>planned_end_at</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>estimated_duration_minutes</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>actual_duration_minutes</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>updated_at</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
@@ -3316,50 +3351,85 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -3389,50 +3459,85 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -3462,50 +3567,85 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -3535,50 +3675,85 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -3608,50 +3783,85 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -3681,50 +3891,85 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -3754,50 +3999,85 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -3827,50 +4107,85 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
         <is>
           <t>8</t>
         </is>
@@ -3900,50 +4215,85 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
         <is>
           <t>9</t>
         </is>
@@ -3973,50 +4323,85 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
         <is>
           <t>10</t>
         </is>
@@ -4046,50 +4431,85 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
         <is>
           <t>11</t>
         </is>
@@ -4119,50 +4539,85 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
         <is>
           <t>12</t>
         </is>
@@ -4192,50 +4647,85 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
         <is>
           <t>13</t>
         </is>
@@ -4265,50 +4755,85 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
         <is>
           <t>14</t>
         </is>
@@ -4338,50 +4863,85 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
         <is>
           <t>15</t>
         </is>
@@ -4411,50 +4971,85 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
         <is>
           <t>16</t>
         </is>
@@ -4484,50 +5079,85 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
         <is>
           <t>17</t>
         </is>
@@ -4557,50 +5187,85 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
         <is>
           <t>18</t>
         </is>
@@ -4630,50 +5295,85 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
         <is>
           <t>19</t>
         </is>
@@ -4703,50 +5403,85 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
         <is>
           <t>20</t>
         </is>
@@ -4776,50 +5511,85 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
         <is>
           <t>21</t>
         </is>
@@ -4849,50 +5619,85 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
         <is>
           <t>22</t>
         </is>
@@ -4922,50 +5727,85 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
         <is>
           <t>23</t>
         </is>
@@ -4995,50 +5835,85 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2030-01-15T07:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ticket_estimate</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
         <is>
           <t>2030-01-15T18:00:00+03:00</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>\N</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>2030-01-15T08:00:00+03:00</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>\N</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>2030-01-15T08:00:00+03:00</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
         <is>
           <t>24</t>
         </is>
@@ -11661,25 +12536,40 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>default_priority</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>travel_minutes</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>work_minutes</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>documents_minutes</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>norm_minutes</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
@@ -11693,25 +12583,40 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>synthetic_1900_1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>15</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>55</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -11725,25 +12630,40 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>synthetic_1900_2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>15</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>55</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -11757,25 +12677,40 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>synthetic_1900_3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>repair</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>15</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>55</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>3</t>
         </is>

</xml_diff>